<commit_message>
MIA: run automatico 2026-09-14 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3892,19 +3892,39 @@
         <v>46276</v>
       </c>
       <c r="B174" t="n">
-        <v>3.99</v>
+        <v>3.990000009536743</v>
       </c>
       <c r="C174" t="n">
-        <v>4.11</v>
+        <v>4.110000133514404</v>
       </c>
       <c r="D174" t="n">
-        <v>3.97</v>
+        <v>3.970000028610229</v>
       </c>
       <c r="E174" t="n">
-        <v>4.02</v>
+        <v>4.019999980926514</v>
       </c>
       <c r="F174" t="n">
         <v>4859300</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B175" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="C175" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="D175" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E175" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="F175" t="n">
+        <v>4246100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-15 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F175"/>
+  <dimension ref="A1:F176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3912,19 +3912,39 @@
         <v>46279</v>
       </c>
       <c r="B175" t="n">
-        <v>4.04</v>
+        <v>4.039999961853027</v>
       </c>
       <c r="C175" t="n">
-        <v>4.07</v>
+        <v>4.070000171661377</v>
       </c>
       <c r="D175" t="n">
-        <v>3.88</v>
+        <v>3.880000114440918</v>
       </c>
       <c r="E175" t="n">
-        <v>3.91</v>
+        <v>3.910000085830688</v>
       </c>
       <c r="F175" t="n">
         <v>4246100</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B176" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="C176" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="D176" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="E176" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F176" t="n">
+        <v>2162200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-16 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F176"/>
+  <dimension ref="A1:F177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3932,19 +3932,39 @@
         <v>46280</v>
       </c>
       <c r="B176" t="n">
-        <v>3.97</v>
+        <v>3.970000028610229</v>
       </c>
       <c r="C176" t="n">
-        <v>4.05</v>
+        <v>4.050000190734863</v>
       </c>
       <c r="D176" t="n">
-        <v>3.96</v>
+        <v>3.960000038146973</v>
       </c>
       <c r="E176" t="n">
-        <v>4.04</v>
+        <v>4.039999961853027</v>
       </c>
       <c r="F176" t="n">
         <v>2162200</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B177" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="C177" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D177" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="E177" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="F177" t="n">
+        <v>4733000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-17 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F177"/>
+  <dimension ref="A1:F178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3952,19 +3952,39 @@
         <v>46281</v>
       </c>
       <c r="B177" t="n">
-        <v>4.11</v>
+        <v>4.110000133514404</v>
       </c>
       <c r="C177" t="n">
-        <v>4.2</v>
+        <v>4.199999809265137</v>
       </c>
       <c r="D177" t="n">
-        <v>3.96</v>
+        <v>3.960000038146973</v>
       </c>
       <c r="E177" t="n">
-        <v>3.98</v>
+        <v>3.980000019073486</v>
       </c>
       <c r="F177" t="n">
         <v>4733000</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B178" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="C178" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="D178" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="E178" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="F178" t="n">
+        <v>4273500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-18 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3972,19 +3972,39 @@
         <v>46282</v>
       </c>
       <c r="B178" t="n">
-        <v>4.18</v>
+        <v>4.179999828338623</v>
       </c>
       <c r="C178" t="n">
-        <v>4.32</v>
+        <v>4.320000171661377</v>
       </c>
       <c r="D178" t="n">
-        <v>4.08</v>
+        <v>4.079999923706055</v>
       </c>
       <c r="E178" t="n">
-        <v>4.15</v>
+        <v>4.150000095367432</v>
       </c>
       <c r="F178" t="n">
         <v>4273500</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B179" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C179" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D179" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="E179" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F179" t="n">
+        <v>4866500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-21 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3992,19 +3992,39 @@
         <v>46283</v>
       </c>
       <c r="B179" t="n">
-        <v>4.2</v>
+        <v>4.199999809265137</v>
       </c>
       <c r="C179" t="n">
-        <v>4.2</v>
+        <v>4.199999809265137</v>
       </c>
       <c r="D179" t="n">
-        <v>4.06</v>
+        <v>4.059999942779541</v>
       </c>
       <c r="E179" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="F179" t="n">
         <v>4866500</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B180" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="C180" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="D180" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="E180" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="F180" t="n">
+        <v>3132600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-22 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F180"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4012,19 +4012,39 @@
         <v>46286</v>
       </c>
       <c r="B180" t="n">
-        <v>4.18</v>
+        <v>4.179999828338623</v>
       </c>
       <c r="C180" t="n">
-        <v>4.29</v>
+        <v>4.289999961853027</v>
       </c>
       <c r="D180" t="n">
-        <v>4.16</v>
+        <v>4.159999847412109</v>
       </c>
       <c r="E180" t="n">
-        <v>4.23</v>
+        <v>4.230000019073486</v>
       </c>
       <c r="F180" t="n">
         <v>3132600</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B181" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="C181" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="D181" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="E181" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="F181" t="n">
+        <v>3875800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-23 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4032,19 +4032,39 @@
         <v>46287</v>
       </c>
       <c r="B181" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="C181" t="n">
-        <v>4.21</v>
+        <v>4.210000038146973</v>
       </c>
       <c r="D181" t="n">
-        <v>4.13</v>
+        <v>4.130000114440918</v>
       </c>
       <c r="E181" t="n">
-        <v>4.14</v>
+        <v>4.139999866485596</v>
       </c>
       <c r="F181" t="n">
         <v>3875800</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B182" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C182" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="D182" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="E182" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="F182" t="n">
+        <v>2664200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-24 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:F183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4052,19 +4052,39 @@
         <v>46288</v>
       </c>
       <c r="B182" t="n">
-        <v>4.2</v>
+        <v>4.199999809265137</v>
       </c>
       <c r="C182" t="n">
-        <v>4.26</v>
+        <v>4.260000228881836</v>
       </c>
       <c r="D182" t="n">
-        <v>4.14</v>
+        <v>4.139999866485596</v>
       </c>
       <c r="E182" t="n">
-        <v>4.16</v>
+        <v>4.159999847412109</v>
       </c>
       <c r="F182" t="n">
         <v>2664200</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B183" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="C183" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="D183" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="E183" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F183" t="n">
+        <v>4885100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-25 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F183"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4072,19 +4072,39 @@
         <v>46289</v>
       </c>
       <c r="B183" t="n">
-        <v>4.08</v>
+        <v>4.079999923706055</v>
       </c>
       <c r="C183" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="D183" t="n">
-        <v>4.01</v>
+        <v>4.010000228881836</v>
       </c>
       <c r="E183" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="F183" t="n">
         <v>4885100</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B184" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="C184" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="D184" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="E184" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1794000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-28 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4092,19 +4092,39 @@
         <v>46290</v>
       </c>
       <c r="B184" t="n">
-        <v>4.09</v>
+        <v>4.090000152587891</v>
       </c>
       <c r="C184" t="n">
-        <v>4.14</v>
+        <v>4.139999866485596</v>
       </c>
       <c r="D184" t="n">
-        <v>4.01</v>
+        <v>4.010000228881836</v>
       </c>
       <c r="E184" t="n">
-        <v>4.08</v>
+        <v>4.079999923706055</v>
       </c>
       <c r="F184" t="n">
         <v>1794000</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B185" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="C185" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="D185" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="E185" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F185" t="n">
+        <v>2754400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-29 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4112,19 +4112,39 @@
         <v>46293</v>
       </c>
       <c r="B185" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="C185" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="D185" t="n">
-        <v>4.01</v>
+        <v>4.010000228881836</v>
       </c>
       <c r="E185" t="n">
-        <v>4.08</v>
+        <v>4.079999923706055</v>
       </c>
       <c r="F185" t="n">
         <v>2754400</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B186" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="C186" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="D186" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="E186" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F186" t="n">
+        <v>1939900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-30 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4132,19 +4132,39 @@
         <v>46294</v>
       </c>
       <c r="B186" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="C186" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="D186" t="n">
-        <v>4.12</v>
+        <v>4.119999885559082</v>
       </c>
       <c r="E186" t="n">
-        <v>4.19</v>
+        <v>4.190000057220459</v>
       </c>
       <c r="F186" t="n">
         <v>1939900</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B187" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="C187" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="D187" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="E187" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F187" t="n">
+        <v>6231900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-01 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F187"/>
+  <dimension ref="A1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4152,19 +4152,39 @@
         <v>46295</v>
       </c>
       <c r="B187" t="n">
-        <v>4.41</v>
+        <v>4.409999847412109</v>
       </c>
       <c r="C187" t="n">
-        <v>4.47</v>
+        <v>4.46999979019165</v>
       </c>
       <c r="D187" t="n">
-        <v>4.21</v>
+        <v>4.210000038146973</v>
       </c>
       <c r="E187" t="n">
         <v>4.25</v>
       </c>
       <c r="F187" t="n">
         <v>6231900</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B188" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="C188" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D188" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E188" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="F188" t="n">
+        <v>5707000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-02 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4172,19 +4172,39 @@
         <v>46296</v>
       </c>
       <c r="B188" t="n">
-        <v>4.47</v>
+        <v>4.5</v>
       </c>
       <c r="C188" t="n">
         <v>4.5</v>
       </c>
       <c r="D188" t="n">
-        <v>4.35</v>
+        <v>4.349999904632568</v>
       </c>
       <c r="E188" t="n">
-        <v>4.44</v>
+        <v>4.440000057220459</v>
       </c>
       <c r="F188" t="n">
         <v>5707000</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B189" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="C189" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="D189" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E189" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="F189" t="n">
+        <v>4954900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-05 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4192,19 +4192,39 @@
         <v>46297</v>
       </c>
       <c r="B189" t="n">
-        <v>4.45</v>
+        <v>4.449999809265137</v>
       </c>
       <c r="C189" t="n">
-        <v>4.58</v>
+        <v>4.579999923706055</v>
       </c>
       <c r="D189" t="n">
-        <v>4.4</v>
+        <v>4.400000095367432</v>
       </c>
       <c r="E189" t="n">
-        <v>4.51</v>
+        <v>4.510000228881836</v>
       </c>
       <c r="F189" t="n">
         <v>4954900</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B190" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="C190" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="D190" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="E190" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="F190" t="n">
+        <v>8939600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-06 22:32 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F190"/>
+  <dimension ref="A1:F191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4215,16 +4215,36 @@
         <v>4.75</v>
       </c>
       <c r="C190" t="n">
-        <v>4.94</v>
+        <v>4.940000057220459</v>
       </c>
       <c r="D190" t="n">
-        <v>4.55</v>
+        <v>4.550000190734863</v>
       </c>
       <c r="E190" t="n">
-        <v>4.69</v>
+        <v>4.690000057220459</v>
       </c>
       <c r="F190" t="n">
         <v>8939600</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B191" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="C191" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D191" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E191" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="F191" t="n">
+        <v>5456900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-07 22:29 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4232,19 +4232,39 @@
         <v>46301</v>
       </c>
       <c r="B191" t="n">
-        <v>4.86</v>
+        <v>4.860000133514404</v>
       </c>
       <c r="C191" t="n">
-        <v>4.9</v>
+        <v>4.900000095367432</v>
       </c>
       <c r="D191" t="n">
-        <v>4.7</v>
+        <v>4.699999809265137</v>
       </c>
       <c r="E191" t="n">
-        <v>4.82</v>
+        <v>4.820000171661377</v>
       </c>
       <c r="F191" t="n">
         <v>5456900</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B192" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="C192" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="D192" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="E192" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="F192" t="n">
+        <v>4142000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-08 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F192"/>
+  <dimension ref="A1:F193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4252,19 +4252,39 @@
         <v>46302</v>
       </c>
       <c r="B192" t="n">
-        <v>4.78</v>
+        <v>4.78000020980835</v>
       </c>
       <c r="C192" t="n">
-        <v>4.94</v>
+        <v>4.940000057220459</v>
       </c>
       <c r="D192" t="n">
-        <v>4.73</v>
+        <v>4.730000019073486</v>
       </c>
       <c r="E192" t="n">
-        <v>4.82</v>
+        <v>4.820000171661377</v>
       </c>
       <c r="F192" t="n">
         <v>4142000</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B193" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="C193" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="D193" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E193" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="F193" t="n">
+        <v>9604200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-09 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F193"/>
+  <dimension ref="A1:F194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4272,19 +4272,39 @@
         <v>46303</v>
       </c>
       <c r="B193" t="n">
-        <v>4.95</v>
+        <v>4.949999809265137</v>
       </c>
       <c r="C193" t="n">
-        <v>5.08</v>
+        <v>5.079999923706055</v>
       </c>
       <c r="D193" t="n">
         <v>4.75</v>
       </c>
       <c r="E193" t="n">
-        <v>4.78</v>
+        <v>4.78000020980835</v>
       </c>
       <c r="F193" t="n">
         <v>9604200</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B194" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="C194" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="D194" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="E194" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="F194" t="n">
+        <v>5269000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-12 22:29 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -4292,16 +4292,16 @@
         <v>46304</v>
       </c>
       <c r="B194" t="n">
-        <v>4.97</v>
+        <v>4.96999979019165</v>
       </c>
       <c r="C194" t="n">
-        <v>5.15</v>
+        <v>5.150000095367432</v>
       </c>
       <c r="D194" t="n">
-        <v>4.91</v>
+        <v>4.909999847412109</v>
       </c>
       <c r="E194" t="n">
-        <v>5.02</v>
+        <v>5.019999980926514</v>
       </c>
       <c r="F194" t="n">
         <v>5269000</v>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-13 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:F195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4307,6 +4307,26 @@
         <v>5269000</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B195" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C195" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="D195" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="E195" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="F195" t="n">
+        <v>4568000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-14 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F195"/>
+  <dimension ref="A1:F196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4312,19 +4312,39 @@
         <v>46308</v>
       </c>
       <c r="B195" t="n">
-        <v>4.9</v>
+        <v>4.900000095367432</v>
       </c>
       <c r="C195" t="n">
-        <v>4.96</v>
+        <v>4.960000038146973</v>
       </c>
       <c r="D195" t="n">
-        <v>4.76</v>
+        <v>4.760000228881836</v>
       </c>
       <c r="E195" t="n">
-        <v>4.95</v>
+        <v>4.949999809265137</v>
       </c>
       <c r="F195" t="n">
         <v>4568000</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B196" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="C196" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="D196" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="E196" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="F196" t="n">
+        <v>3225700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-15 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F196"/>
+  <dimension ref="A1:F197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4332,19 +4332,39 @@
         <v>46309</v>
       </c>
       <c r="B196" t="n">
-        <v>4.92</v>
+        <v>4.920000076293945</v>
       </c>
       <c r="C196" t="n">
-        <v>4.94</v>
+        <v>4.929999828338623</v>
       </c>
       <c r="D196" t="n">
-        <v>4.73</v>
+        <v>4.730000019073486</v>
       </c>
       <c r="E196" t="n">
-        <v>4.88</v>
+        <v>4.880000114440918</v>
       </c>
       <c r="F196" t="n">
         <v>3225700</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B197" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="C197" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="D197" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="E197" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="F197" t="n">
+        <v>7769900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-16 22:29 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F197"/>
+  <dimension ref="A1:F198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4352,19 +4352,39 @@
         <v>46310</v>
       </c>
       <c r="B197" t="n">
-        <v>5.01</v>
+        <v>5.010000228881836</v>
       </c>
       <c r="C197" t="n">
-        <v>5.19</v>
+        <v>5.190000057220459</v>
       </c>
       <c r="D197" t="n">
-        <v>4.81</v>
+        <v>4.809999942779541</v>
       </c>
       <c r="E197" t="n">
-        <v>4.83</v>
+        <v>4.829999923706055</v>
       </c>
       <c r="F197" t="n">
         <v>7769900</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B198" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="C198" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="D198" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="E198" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="F198" t="n">
+        <v>8656200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-19 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F198"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4372,19 +4372,39 @@
         <v>46311</v>
       </c>
       <c r="B198" t="n">
-        <v>5.07</v>
+        <v>5.070000171661377</v>
       </c>
       <c r="C198" t="n">
-        <v>5.18</v>
+        <v>5.179999828338623</v>
       </c>
       <c r="D198" t="n">
-        <v>4.89</v>
+        <v>4.889999866485596</v>
       </c>
       <c r="E198" t="n">
-        <v>5.04</v>
+        <v>5.039999961853027</v>
       </c>
       <c r="F198" t="n">
-        <v>8656200</v>
+        <v>8655200</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B199" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="C199" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D199" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="E199" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="F199" t="n">
+        <v>3793000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-20 22:29 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F199"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4392,19 +4392,39 @@
         <v>46314</v>
       </c>
       <c r="B199" t="n">
-        <v>5.09</v>
+        <v>5.090000152587891</v>
       </c>
       <c r="C199" t="n">
-        <v>5.2</v>
+        <v>5.199999809265137</v>
       </c>
       <c r="D199" t="n">
-        <v>5.05</v>
+        <v>5.050000190734863</v>
       </c>
       <c r="E199" t="n">
-        <v>5.08</v>
+        <v>5.079999923706055</v>
       </c>
       <c r="F199" t="n">
         <v>3793000</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B200" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="C200" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="D200" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="E200" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="F200" t="n">
+        <v>7869900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-21 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4412,19 +4412,39 @@
         <v>46315</v>
       </c>
       <c r="B200" t="n">
-        <v>5.26</v>
+        <v>5.260000228881836</v>
       </c>
       <c r="C200" t="n">
-        <v>5.32</v>
+        <v>5.320000171661377</v>
       </c>
       <c r="D200" t="n">
-        <v>5.09</v>
+        <v>5.090000152587891</v>
       </c>
       <c r="E200" t="n">
-        <v>5.12</v>
+        <v>5.119999885559082</v>
       </c>
       <c r="F200" t="n">
         <v>7869900</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B201" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="C201" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="D201" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="E201" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="F201" t="n">
+        <v>3635100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-22 23:58 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4432,19 +4432,39 @@
         <v>46316</v>
       </c>
       <c r="B201" t="n">
-        <v>5.31</v>
+        <v>5.309999942779541</v>
       </c>
       <c r="C201" t="n">
-        <v>5.37</v>
+        <v>5.369999885559082</v>
       </c>
       <c r="D201" t="n">
-        <v>5.17</v>
+        <v>5.170000076293945</v>
       </c>
       <c r="E201" t="n">
-        <v>5.29</v>
+        <v>5.289999961853027</v>
       </c>
       <c r="F201" t="n">
         <v>3635100</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B202" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="C202" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="D202" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="E202" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="F202" t="n">
+        <v>4088000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-23 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F202"/>
+  <dimension ref="A1:F203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4452,19 +4452,39 @@
         <v>46317</v>
       </c>
       <c r="B202" t="n">
-        <v>5.17</v>
+        <v>5.170000076293945</v>
       </c>
       <c r="C202" t="n">
-        <v>5.28</v>
+        <v>5.28000020980835</v>
       </c>
       <c r="D202" t="n">
-        <v>5.07</v>
+        <v>5.070000171661377</v>
       </c>
       <c r="E202" t="n">
-        <v>5.24</v>
+        <v>5.239999771118164</v>
       </c>
       <c r="F202" t="n">
         <v>4088000</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B203" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="C203" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="D203" t="n">
+        <v>5</v>
+      </c>
+      <c r="E203" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F203" t="n">
+        <v>6215400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-26 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F203"/>
+  <dimension ref="A1:F204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4472,19 +4472,39 @@
         <v>46318</v>
       </c>
       <c r="B203" t="n">
-        <v>5.28</v>
+        <v>5.28000020980835</v>
       </c>
       <c r="C203" t="n">
-        <v>5.32</v>
+        <v>5.320000171661377</v>
       </c>
       <c r="D203" t="n">
         <v>5</v>
       </c>
       <c r="E203" t="n">
-        <v>5.2</v>
+        <v>5.199999809265137</v>
       </c>
       <c r="F203" t="n">
         <v>6215400</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B204" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="C204" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="D204" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="E204" t="n">
+        <v>4</v>
+      </c>
+      <c r="F204" t="n">
+        <v>17478500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-27 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F204"/>
+  <dimension ref="A1:F205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4492,19 +4492,39 @@
         <v>46321</v>
       </c>
       <c r="B204" t="n">
-        <v>4.11</v>
+        <v>4.110000133514404</v>
       </c>
       <c r="C204" t="n">
-        <v>4.11</v>
+        <v>4.110000133514404</v>
       </c>
       <c r="D204" t="n">
-        <v>3.73</v>
+        <v>3.730000019073486</v>
       </c>
       <c r="E204" t="n">
         <v>4</v>
       </c>
       <c r="F204" t="n">
         <v>17478500</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B205" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="C205" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="D205" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="E205" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="F205" t="n">
+        <v>14606200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-28 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F205"/>
+  <dimension ref="A1:F206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4512,19 +4512,39 @@
         <v>46322</v>
       </c>
       <c r="B205" t="n">
-        <v>4.12</v>
+        <v>4.119999885559082</v>
       </c>
       <c r="C205" t="n">
-        <v>4.23</v>
+        <v>4.230000019073486</v>
       </c>
       <c r="D205" t="n">
-        <v>4.03</v>
+        <v>4.039999961853027</v>
       </c>
       <c r="E205" t="n">
-        <v>4.14</v>
+        <v>4.139999866485596</v>
       </c>
       <c r="F205" t="n">
         <v>14606200</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B206" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C206" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="D206" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E206" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F206" t="n">
+        <v>6441300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-10-29 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F206"/>
+  <dimension ref="A1:F207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4532,19 +4532,39 @@
         <v>46323</v>
       </c>
       <c r="B206" t="n">
-        <v>3.95</v>
+        <v>3.950000047683716</v>
       </c>
       <c r="C206" t="n">
-        <v>4.12</v>
+        <v>4.119999885559082</v>
       </c>
       <c r="D206" t="n">
-        <v>3.78</v>
+        <v>3.789999961853027</v>
       </c>
       <c r="E206" t="n">
-        <v>4.12</v>
+        <v>4.119999885559082</v>
       </c>
       <c r="F206" t="n">
         <v>6441300</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B207" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="C207" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="D207" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="E207" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="F207" t="n">
+        <v>3042400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>